<commit_message>
feat(dataiq): descripción del instrumental en la carga inicial
La hoja catalogo de seed/tecnicas.xlsx suma las columnas alias, descripcion
y fuentes_descripcion, con la descripción de los 23 instrumentos de la mesa
de Mayo de Cirugía General y sus fuentes. La carga llena la descripción solo
si el instrumento no tiene una, y renombra sin cambiar el id cuando el nombre
anterior viene como alias (Pinza Moninjan -> Pinza de Moynihan).
</commit_message>
<xml_diff>
--- a/dataiq/backend/seed/tecnicas.xlsx
+++ b/dataiq/backend/seed/tecnicas.xlsx
@@ -589,7 +589,7 @@
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>Solo consulta: el catálogo de instrumental de DataIQ.</t>
+          <t>El catálogo de instrumental: categoría y nombre; alias = nombres anteriores o variantes, separados por ';'; descripcion = lo que ve el estudiante al tocar el instrumento; fuentes_descripcion = una fuente por línea. La carga llena la descripción solo si el instrumento no tiene una.</t>
         </is>
       </c>
     </row>
@@ -9093,7 +9093,7 @@
       </c>
       <c r="E9" s="6" t="inlineStr">
         <is>
-          <t>Pinza Moninjan</t>
+          <t>Pinza de Moynihan</t>
         </is>
       </c>
       <c r="F9" s="6" t="inlineStr">
@@ -12977,7 +12977,7 @@
       </c>
       <c r="E125" s="6" t="inlineStr">
         <is>
-          <t>Pinza Moninjan</t>
+          <t>Pinza de Moynihan</t>
         </is>
       </c>
       <c r="F125" s="6" t="inlineStr"/>
@@ -24500,7 +24500,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B144"/>
+  <dimension ref="A1:E144"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -24518,6 +24518,21 @@
           <t>nombre</t>
         </is>
       </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>alias</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>descripcion</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>fuentes_descripcion</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
@@ -24734,6 +24749,17 @@
           <t>Mango de bisturí N.° 3</t>
         </is>
       </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Mango de acero inoxidable, de un solo cuerpo, en el que se monta la hoja de bisturí. El número indica la forma del extremo donde encaja la hoja: el N.° 3 recibe las hojas pequeñas (N.° 10, 11, 12 y 15). Es instrumental de diéresis: con la hoja montada, sirve para hacer las incisiones.</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>CICR, XSINMEDI012703, mango N.° 3 para hojas 10/11/15: https://itemscatalogue.redcross.int/detail.aspx?itemcode=XSINMEDI012703&amp;from=kit
+Sánchez-Sarría O. y otros, Manual de instrumental quirúrgico, Medisur 2014;12(5), p. 783: https://medisur.sld.cu/index.php/medisur/article/view/2662</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="5" t="inlineStr">
@@ -24746,6 +24772,17 @@
           <t>Mango de bisturí N.° 4</t>
         </is>
       </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Mango de acero inoxidable, de un solo cuerpo, en el que se monta la hoja de bisturí. Recibe las hojas grandes (N.° 20, 21 y 22). Es instrumental de diéresis: con la hoja montada, sirve para hacer las incisiones.</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>CICR, set KMSISBAS01, mango N.° 4 para hojas 20: https://itemscatalogue.redcross.int/detail.aspx?itemcode=KMSISBAS01&amp;from=kit
+Sánchez-Sarría O. y otros, Manual de instrumental quirúrgico, Medisur 2014;12(5), p. 783: https://medisur.sld.cu/index.php/medisur/article/view/2662</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="6" t="inlineStr">
@@ -24758,6 +24795,19 @@
           <t>Mango de bisturí N.° 7</t>
         </is>
       </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Mango de bisturí más largo y delgado que el N.° 3. Recibe las mismas hojas pequeñas (N.° 10, 11, 12 y 15). Su vástago delgado permite incisiones finas y precisas en espacios reducidos o en planos profundos. Mide unos 16 cm.</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Sánchez-Sarría O. y otros, Manual de instrumental quirúrgico, Medisur 2014;12(5), p. 783: https://medisur.sld.cu/index.php/medisur/article/view/2662
+Bard-Parker (Aspen Surgical), mango N.° 7, en VWR: https://b2b-us.vwr.com/store/product/4636508/null
+Sklar 97-042, en McKesson: https://mms.mckesson.com/product/368400/Sklar-97-042
+V. Mueller, registro GUDID (NLM): https://accessgudid.nlm.nih.gov/devices/10885403059599</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
@@ -25022,6 +25072,17 @@
           <t>Pinza de Allis</t>
         </is>
       </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>Pinza de aprehensión con anillos y cremallera, que se queda cerrada sobre el tejido. Sus mandíbulas terminan en varios dientes finos que encajan entre sí (4 × 5 en el modelo estándar). Sirve para tomar y mantener sujetos tejidos y estructuras durante la operación. Mide de 14 a 20 cm.</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>CICR, XSINMEDI500215, pinza de Allis: https://itemscatalogue.redcross.int/detail.aspx?itemcode=XSINMEDI500215&amp;from=kit
+Sánchez-Sarría O. y otros, Manual de instrumental quirúrgico, Medisur 2014;12(5), p. 784: https://medisur.sld.cu/index.php/medisur/article/view/2662</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="5" t="inlineStr">
@@ -25034,6 +25095,18 @@
           <t>Pinza de Babcock</t>
         </is>
       </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>Pinza de aprehensión con anillos y cremallera suave. Su punta es ancha, redondeada y abierta en el centro (fenestrada), sin dientes, con estrías atraumáticas. Toma tejidos blandos y delicados, sobre todo el intestino, sin aplastarlos ni perforarlos. Es más suave con el tejido que la pinza de Allis. Mide de 16 a 21 cm.</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>UNICEF Supply Catalogue, S0736500, Babcock 200 mm (ref. KLS Martin 30 192 20): https://supply.unicef.org/s0736500.html
+KLS Martin, 30-196-20-07: https://www.klsmartin.com/shop/en/products/product/30-196-20-07/
+Eickemeyer, 145616: https://www.eickemeyer.com/shop/145616-intestinal-and-tissue-forceps-babcock-16-cm-atraumatic-13535</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="6" t="inlineStr">
@@ -25130,6 +25203,18 @@
           <t>Pinza de disección con garra</t>
         </is>
       </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>Pinza de un solo cuerpo, de resorte y sin cremallera, como la de disección sin garra, pero con dientes en la punta. Los dientes de las dos ramas encajan entre sí: uno en una rama entre dos de la otra («1 × 2»). Así agarra con más firmeza que la sin garra. Mide de 14 a 20 cm.</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>CICR, XSINMEDI060020, pinza de disección 1 × 2 dientes (XSINMEDI060520): https://itemscatalogue.redcross.int/detail.aspx?itemcode=XSINMEDI060020&amp;from=kit
+Sánchez-Sarría O. y otros, Manual de instrumental quirúrgico, Medisur 2014;12(5), p. 784: https://medisur.sld.cu/index.php/medisur/article/view/2662
+UNAM, Facultad de Medicina, Práctica 3: estuche de disección (2023): https://anatomia.facmed.unam.mx/wp-content/uploads/2023/10/Practica-3-estuche-2023-2024.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="6" t="inlineStr">
@@ -25142,6 +25227,18 @@
           <t>Pinza de disección sin garra</t>
         </is>
       </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>Pinza de un solo cuerpo, de resorte: se cierra al presionar sus ramas y se abre sola al soltarlas. No tiene cremallera. Sus puntas son estriadas y no tienen dientes, por eso no lastiman el tejido. Sirve para tomar tejidos delicados durante la disección y la sutura, y para manipular gasas y apósitos. Mide de 14,5 a 20 cm.</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>CICR, XSINMEDI060020, pinza de disección con o sin dientes: https://itemscatalogue.redcross.int/detail.aspx?itemcode=XSINMEDI060020&amp;from=kit
+Sánchez-Sarría O. y otros, Manual de instrumental quirúrgico, Medisur 2014;12(5), p. 784: https://medisur.sld.cu/index.php/medisur/article/view/2662
+UNAM, Facultad de Medicina, Práctica 3: estuche de disección (2023): https://anatomia.facmed.unam.mx/wp-content/uploads/2023/10/Practica-3-estuche-2023-2024.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="5" t="inlineStr">
@@ -25202,6 +25299,20 @@
           <t>Pinza Kelly</t>
         </is>
       </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>Pinza hemostática con anillos y cremallera, recta o curva, de unos 14 cm. Sus mandíbulas tienen estrías transversales solo en la mitad de la punta; eso la distingue de la pinza Crile, que es estriada en toda la mandíbula. Sirve para pinzar vasos o tejidos y así evitar la hemorragia.</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>UNAM, Facultad de Medicina, Práctica 3: estuche de disección (2023): https://anatomia.facmed.unam.mx/wp-content/uploads/2023/10/Practica-3-estuche-2023-2024.pdf
+Sánchez-Sarría O. y otros, Manual de instrumental quirúrgico, Medisur 2014;12(5), p. 784: https://medisur.sld.cu/index.php/medisur/article/view/2662
+MSF Unicat 14066, Kelly 14 cm: https://unicat.msf.org/cat/product/14066
+Remma, Kelly 14 cm: https://remma.fr/en/model/kelly-clamp-straight-curved-jaws-serrated-14-cm
+Medikabazaar, guía de la pinza Kelly: https://www.medikabazaar.com/blogs/kelly-forceps-types-uses-surgical-procurement-guide</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="6" t="inlineStr">
@@ -25214,6 +25325,18 @@
           <t>Pinza Kelly Adson</t>
         </is>
       </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>Pinza hemostática de Adson, con anillos y cremallera, recta o curva, de unos 18 cm. Sus ramas son más largas que las de la Kelly y sus mandíbulas, estriadas en parte. Sirve para pinzar vasos pequeños. No es la pinza de disección Adson, que es de aprehensión.</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>Sánchez-Sarría O. y otros, Manual de instrumental quirúrgico, Medisur 2014;12(5), p. 784: https://medisur.sld.cu/index.php/medisur/article/view/2662
+Sklar 50-1372, Adson hemostática recta, en McKesson: https://mms.mckesson.com/product/253068/Sklar-50-1372
+Sklar 50-1472, Adson hemostática curva, en McKesson: https://mms.mckesson.com/product/377086/Sklar-50-1472</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="5" t="inlineStr">
@@ -25226,6 +25349,17 @@
           <t>Pinza Kocher</t>
         </is>
       </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>Pinza hemostática con anillos y cremallera, recta o curva, de 14 a 22 cm. Sus mandíbulas son estriadas y terminan en dientes (1 × 2: uno en una rama entre dos de la otra). Sirve para hemostasia, para sujetar tejidos y para sostener gasas.</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>CICR, XSINMEDI161214, Kocher y R-Ochsner: https://itemscatalogue.redcross.int/detail.aspx?itemcode=XSINMEDI161214&amp;from=kit
+Sánchez-Sarría O. y otros, Manual de instrumental quirúrgico, Medisur 2014;12(5), p. 786: https://medisur.sld.cu/index.php/medisur/article/view/2662</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="6" t="inlineStr">
@@ -25247,7 +25381,23 @@
       </c>
       <c r="B62" s="5" t="inlineStr">
         <is>
+          <t>Pinza de Moynihan</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
           <t>Pinza Moninjan</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>Pinza larga y curva, de unos 22 a 23 cm, con anillos, hecha para tomar el conducto biliar. Sus mandíbulas son estriadas.</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>KLS Martin, 13-671-23-07, bile duct forceps acc. to Moynihan: https://www.klsmartin.com/shop/en/products/product/13-671-23-07/
+Ambler Surgical 32-444, registro FDA (UDI 00190660066611): https://beudamed.com/fda_udis/00190660066611</t>
         </is>
       </c>
     </row>
@@ -25262,6 +25412,18 @@
           <t>Pinza Mosquito curva</t>
         </is>
       </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>Pinza hemostática pequeña y delgada (de Halsted), de unos 12,5 cm, con anillos y cremallera. Sus mandíbulas son finas y curvas. Sirve para pinzar vasos pequeños, para disecciones finas y para tomar tejidos delicados.</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>CICR, XSINMEDI154512, H-Mosquito curva: https://itemscatalogue.redcross.int/detail.aspx?itemcode=XSINMEDI154512&amp;from=kit
+UNAM, Facultad de Medicina, Práctica 3: estuche de disección (2023): https://anatomia.facmed.unam.mx/wp-content/uploads/2023/10/Practica-3-estuche-2023-2024.pdf
+Sánchez-Sarría O. y otros, Manual de instrumental quirúrgico, Medisur 2014;12(5), p. 784: https://medisur.sld.cu/index.php/medisur/article/view/2662</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="5" t="inlineStr">
@@ -25286,6 +25448,19 @@
           <t>Pinza Rochester</t>
         </is>
       </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>Pinza hemostática grande y fuerte (Rochester-Péan), con anillos y cremallera, recta o curva, de 16 a 26 cm. Sus mandíbulas tienen estrías transversales en todo su largo. Sirve para pinzar tejidos gruesos y vasos grandes.</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>Sánchez-Sarría O. y otros, Manual de instrumental quirúrgico, Medisur 2014;12(5), p. 784: https://medisur.sld.cu/index.php/medisur/article/view/2662
+MSF Unicat 14060, R-Pean 16 cm: https://unicat.msf.org/cat/product/14060
+Covetrus, Rochester-Pean: https://products.covetrus.com/surgical-instruments/forceps-hemostats/hemostat-forceps-rochester-pean
+UNFPA, 1000326, Rochester-Pean 22 cm: https://globalsupply.unfpa.org/products/forceps-artery-rochester-pean-22cm-straight-1000326.html</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="5" t="inlineStr">
@@ -25334,6 +25509,17 @@
           <t>Portaagujas largo</t>
         </is>
       </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>Portaagujas (Mayo-Hegar) con anillos y cremallera: sostiene la aguja mientras se sutura. Sus mandíbulas tienen estrías marcadas, para agujas estándar, y una ranura a lo largo que evita dañar la aguja. La cremallera deja ajustar la presión. El largo mide de 18 a 23 cm; el corriente, 15 cm.</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>CICR, XSINMEDI101815, portaagujas Mayo-Hegar: https://itemscatalogue.redcross.int/detail.aspx?itemcode=XSINMEDI101815&amp;from=kit
+Sánchez-Sarría O. y otros, Manual de instrumental quirúrgico, Medisur 2014;12(5), p. 784: https://medisur.sld.cu/index.php/medisur/article/view/2662</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="5" t="inlineStr">
@@ -25466,6 +25652,18 @@
           <t>Separador de Farabeuf</t>
         </is>
       </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>Separador manual, de un solo cuerpo, de doble extremo: en cada punta tiene una lámina plana doblada en ángulo recto, de distinto tamaño (24 × 16 y 28 × 16 mm). Mide unos 15 cm y se usa en pares. Retrae la piel, el tejido subcutáneo y el músculo para que el cirujano vea el campo operatorio.</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>CICR, XSINMEDI221015, Farabeuf: https://itemscatalogue.redcross.int/health--3/surgical-instruments--24/surgical-instruments--111/retractor-general-double-ended-farabeuf-roux-senn-miller--XSINMEDI200.aspx
+UNAM, Facultad de Medicina, Práctica 3: estuche de disección (2023): https://anatomia.facmed.unam.mx/wp-content/uploads/2023/10/Practica-3-estuche-2023-2024.pdf
+Sánchez-Sarría O. y otros, Manual de instrumental quirúrgico, Medisur 2014;12(5), p. 783: https://medisur.sld.cu/index.php/medisur/article/view/2662</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="6" t="inlineStr">
@@ -25490,6 +25688,19 @@
           <t>Separador de Senn Miller</t>
         </is>
       </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>Separador manual pequeño, de doble extremo: en un extremo tiene tres puntas curvas (romas o agudas) y en el otro, una lámina delgada doblada. Mide unos 15 a 16 cm. Retrae la piel, el tejido o el músculo en sitios quirúrgicos pequeños.</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>CICR, XSINMEDI200509, Senn-Miller: https://itemscatalogue.redcross.int/health--3/surgical-instruments--24/surgical-instruments--111/retractor-general-double-ended-farabeuf-roux-senn-miller--XSINMEDI200.aspx
+Sklar, Miller-Senn, en VWR: https://b2b-pr.vwr.com/store/product/18360095/null
+Sklar Senn, en Ward's Science: https://www.wardsci.com/us/en/product/NA1063474/senn-retractor-or-grade-sklar
+Sánchez-Sarría O. y otros, Manual de instrumental quirúrgico, Medisur 2014;12(5), p. 783: https://medisur.sld.cu/index.php/medisur/article/view/2662</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="6" t="inlineStr">
@@ -25766,6 +25977,17 @@
           <t>Hoja de bisturí #10</t>
         </is>
       </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>Hoja de bisturí pequeña, de acero, con el filo curvo, que se monta en los mangos N.° 3 y N.° 7. Es la forma clásica para las incisiones en piel y músculo.</t>
+        </is>
+      </c>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>Sánchez-Sarría O. y otros, Manual de instrumental quirúrgico, Medisur 2014;12(5), p. 783: https://medisur.sld.cu/index.php/medisur/article/view/2662
+Swann-Morton, hojas de bisturí (IMS Euro): https://imseuro.co.uk/swann-mortonr-scalpel-blades</t>
+        </is>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="5" t="inlineStr">
@@ -25778,6 +26000,17 @@
           <t>Hoja de bisturí #10-11</t>
         </is>
       </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>Hojas pequeñas N.° 10 y N.° 11, que se montan en el mango N.° 3. La N.° 10 tiene el filo curvo y es la forma clásica para incisiones en piel y músculo. La N.° 11 es triangular, con la punta aguda y el filo en uno de sus lados largos: sirve para incisiones punzantes, como abrir un absceso o el sitio de un dren.</t>
+        </is>
+      </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>Sánchez-Sarría O. y otros, Manual de instrumental quirúrgico, Medisur 2014;12(5), p. 783: https://medisur.sld.cu/index.php/medisur/article/view/2662
+Swann-Morton, hojas de bisturí (IMS Euro): https://imseuro.co.uk/swann-mortonr-scalpel-blades</t>
+        </is>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="6" t="inlineStr">
@@ -25802,6 +26035,17 @@
           <t>Hoja de bisturí #15</t>
         </is>
       </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>Hoja de bisturí pequeña, con el filo curvo y corto, que se monta en los mangos N.° 3 y N.° 7. Es la forma más usada para incisiones cortas y precisas.</t>
+        </is>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>Sánchez-Sarría O. y otros, Manual de instrumental quirúrgico, Medisur 2014;12(5), p. 783: https://medisur.sld.cu/index.php/medisur/article/view/2662
+Swann-Morton, hojas de bisturí (IMS Euro): https://imseuro.co.uk/swann-mortonr-scalpel-blades</t>
+        </is>
+      </c>
     </row>
     <row r="109">
       <c r="A109" s="6" t="inlineStr">
@@ -25814,6 +26058,18 @@
           <t>Hoja de bisturí #20</t>
         </is>
       </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>Hoja de bisturí grande, que se monta en el mango N.° 4. Es como una N.° 10 de mayor tamaño: filo curvo y lomo recto sin filo.</t>
+        </is>
+      </c>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>Sánchez-Sarría O. y otros, Manual de instrumental quirúrgico, Medisur 2014;12(5), p. 783: https://medisur.sld.cu/index.php/medisur/article/view/2662
+CICR, set KMSISBAS01, mango N.° 4 para hojas 20: https://itemscatalogue.redcross.int/detail.aspx?itemcode=KMSISBAS01&amp;from=kit
+Swann-Morton N.° 20, en Scientific Laboratory Supplies: https://scientificlabs.co.uk/product/scalpels-and-blades/INS4680</t>
+        </is>
+      </c>
     </row>
     <row r="110">
       <c r="A110" s="5" t="inlineStr">
@@ -26006,6 +26262,18 @@
           <t>Pinza Lahey</t>
         </is>
       </c>
+      <c r="D125" t="inlineStr">
+        <is>
+          <t>Pinza de tracción con anillos y cremallera. Sus puntas son curvas y tienen tres dientes agudos en cada rama (3 × 3), que penetran el tejido fibroso para que el agarre no se suelte. Se usa para tomar y traccionar el tejido y la glándula en la cirugía de tiroides, y el tejido mamario en la mastectomía. Mide unos 15 a 16 cm.</t>
+        </is>
+      </c>
+      <c r="E125" t="inlineStr">
+        <is>
+          <t>Sklar 17-3562, en McKesson: https://mms.mckesson.com/product/375723/Sklar-17-3562
+Aspen Surgical 73-7233, Lahey Goiter Traction 3x3: https://www.mymapmedical.com/shop/aspen-surgical-73-7233-180067
+Integra Miltex 7-62, en McKesson: https://mms.mckesson.com/product/263612/Integra-Lifesciences-7-62</t>
+        </is>
+      </c>
     </row>
     <row r="126">
       <c r="A126" s="5" t="inlineStr">
@@ -26174,6 +26442,17 @@
           <t>Tijera de Mayo</t>
         </is>
       </c>
+      <c r="D139" t="inlineStr">
+        <is>
+          <t>Tijera fuerte, de hojas gruesas y puntas romas, recta o curva, de 15 a 23 cm. Corta por cizalla. La recta se usa para cortar suturas, gasas y otros materiales; la curva también corta tejido que no es delicado.</t>
+        </is>
+      </c>
+      <c r="E139" t="inlineStr">
+        <is>
+          <t>CICR, XSINMEDI035117, tijera de Mayo: https://itemscatalogue.redcross.int/detail.aspx?itemcode=XSINMEDI035117&amp;from=kit
+Sánchez-Sarría O. y otros, Manual de instrumental quirúrgico, Medisur 2014;12(5), p. 783: https://medisur.sld.cu/index.php/medisur/article/view/2662</t>
+        </is>
+      </c>
     </row>
     <row r="140">
       <c r="A140" s="5" t="inlineStr">
@@ -26184,6 +26463,17 @@
       <c r="B140" s="5" t="inlineStr">
         <is>
           <t>Tijera de Metzenbaum</t>
+        </is>
+      </c>
+      <c r="D140" t="inlineStr">
+        <is>
+          <t>Tijera delgada, de puntas romas, casi siempre curva, de 14 a 23 cm. Es la tijera para la disección fina de los tejidos; el material (suturas, gasas) se corta con la tijera de Mayo.</t>
+        </is>
+      </c>
+      <c r="E140" t="inlineStr">
+        <is>
+          <t>CICR, XSINMEDI043318, tijera de Metzenbaum: https://itemscatalogue.redcross.int/detail.aspx?itemcode=XSINMEDI043318&amp;from=kit
+Sánchez-Sarría O. y otros, Manual de instrumental quirúrgico, Medisur 2014;12(5), p. 783: https://medisur.sld.cu/index.php/medisur/article/view/2662</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix(dataiq): descripciones revisadas contra sus fuentes
Cada frase de las 23 descripciones se comparó con la página que la cita.
Salen las que la fuente no decía y las fuentes que no se pueden abrir
(UNICEF, VWR, IMS Euro, McKesson); entran el CICR, JOMI, Swann-Morton y la
guía de HSPA CIS. La Moynihan se describe por su forma, porque también está
en Tiroidectomía, y la Lahey con sus dos versiones.
</commit_message>
<xml_diff>
--- a/dataiq/backend/seed/tecnicas.xlsx
+++ b/dataiq/backend/seed/tecnicas.xlsx
@@ -589,7 +589,7 @@
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>El catálogo de instrumental: categoría y nombre; alias = nombres anteriores o variantes, separados por ';'; descripcion = lo que ve el estudiante al tocar el instrumento; fuentes_descripcion = una fuente por línea. La carga llena la descripción solo si el instrumento no tiene una.</t>
+          <t>El catálogo de instrumental: categoría y nombre; alias = nombres anteriores o variantes, separados por ';'; descripcion = lo que ve el estudiante al tocar el instrumento; fuentes_descripcion = una fuente por línea (va a instruments.description_source). La carga llena la descripción solo si el instrumento no tiene una; con --descriptions reemplaza las que son distintas.</t>
         </is>
       </c>
     </row>
@@ -24756,8 +24756,9 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>CICR, XSINMEDI012703, mango N.° 3 para hojas 10/11/15: https://itemscatalogue.redcross.int/detail.aspx?itemcode=XSINMEDI012703&amp;from=kit
-Sánchez-Sarría O. y otros, Manual de instrumental quirúrgico, Medisur 2014;12(5), p. 783: https://medisur.sld.cu/index.php/medisur/article/view/2662</t>
+          <t>CICR, XSINMEDI0127, mango N.° 3 para hojas 10/11/15: https://itemscatalogue.redcross.int/health--3/surgical-instruments--24/surgical-instruments--111/scalpel-handle-no3--XSINMEDI0127.aspx
+Sánchez-Sarría O. y otros, Manual de instrumental quirúrgico, Medisur 2014;12(5), p. 783: https://medisur.sld.cu/index.php/medisur/article/view/2662
+Open Exam Prep, HSPA CIS, 1.4 Cutting &amp; Dissecting Instruments: https://open-exam-prep.com/study-guides/hspa-cis/instrument-identification/cutting-dissecting</t>
         </is>
       </c>
     </row>
@@ -24774,13 +24775,15 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Mango de acero inoxidable, de un solo cuerpo, en el que se monta la hoja de bisturí. Recibe las hojas grandes (N.° 20, 21 y 22). Es instrumental de diéresis: con la hoja montada, sirve para hacer las incisiones.</t>
+          <t>Mango de acero inoxidable, de un solo cuerpo, en el que se monta la hoja de bisturí. Recibe las hojas grandes (N.° 20, 21 y 22), que no encajan en el N.° 3. Con la hoja montada, sirve para las incisiones grandes.</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>CICR, set KMSISBAS01, mango N.° 4 para hojas 20: https://itemscatalogue.redcross.int/detail.aspx?itemcode=KMSISBAS01&amp;from=kit
-Sánchez-Sarría O. y otros, Manual de instrumental quirúrgico, Medisur 2014;12(5), p. 783: https://medisur.sld.cu/index.php/medisur/article/view/2662</t>
+          <t>CICR, XSINMEDI0128, mango N.° 4 para hojas 20 y 22: https://itemscatalogue.redcross.int/health--3/surgical-instruments--24/surgical-instruments--111/scalpel-handle-no4--XSINMEDI0128.aspx
+Sánchez-Sarría O. y otros, Manual de instrumental quirúrgico, Medisur 2014;12(5), p. 783: https://medisur.sld.cu/index.php/medisur/article/view/2662
+Buckner B., Scalpels, Journal of Medical Insight (JOMI) 300.1, 2023, doi:10.24296/jomi/300.1: https://jomi.com/article/300.1/scalpels/transcript
+Open Exam Prep, HSPA CIS, 1.4 Cutting &amp; Dissecting Instruments: https://open-exam-prep.com/study-guides/hspa-cis/instrument-identification/cutting-dissecting</t>
         </is>
       </c>
     </row>
@@ -24797,15 +24800,17 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Mango de bisturí más largo y delgado que el N.° 3. Recibe las mismas hojas pequeñas (N.° 10, 11, 12 y 15). Su vástago delgado permite incisiones finas y precisas en espacios reducidos o en planos profundos. Mide unos 16 cm.</t>
+          <t>Mango de bisturí largo y delgado. Recibe las mismas hojas pequeñas que el N.° 3 (N.° 10, 11, 12 y 15). Sirve para trabajos finos en planos profundos; su uso más común es con la hoja N.° 11, para hacer una punción. Mide de 15 a 16 cm.</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
           <t>Sánchez-Sarría O. y otros, Manual de instrumental quirúrgico, Medisur 2014;12(5), p. 783: https://medisur.sld.cu/index.php/medisur/article/view/2662
-Bard-Parker (Aspen Surgical), mango N.° 7, en VWR: https://b2b-us.vwr.com/store/product/4636508/null
-Sklar 97-042, en McKesson: https://mms.mckesson.com/product/368400/Sklar-97-042
-V. Mueller, registro GUDID (NLM): https://accessgudid.nlm.nih.gov/devices/10885403059599</t>
+Buckner B., Scalpels, Journal of Medical Insight (JOMI) 300.1, 2023, doi:10.24296/jomi/300.1: https://jomi.com/article/300.1/scalpels/transcript
+Open Exam Prep, HSPA CIS, 1.4 Cutting &amp; Dissecting Instruments: https://open-exam-prep.com/study-guides/hspa-cis/instrument-identification/cutting-dissecting
+Swann-Morton, mango N.° 7, en DD Group: https://ddgroup.com/surgical--implantology/scalpels/shs035--scalpel-handle-stainless-steel---no.7-0907
+V. Mueller SU1407, registro GUDID (FDA): https://accessgudid.nlm.nih.gov/devices/10885403059599
+UNFPA, 1000663, mango N.° 7 de 15 cm: https://globalsupply.unfpa.org/products/scalpel-handle-no-7-blade-holder-15-cm-1000663.html</t>
         </is>
       </c>
     </row>
@@ -25074,12 +25079,13 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Pinza de aprehensión con anillos y cremallera, que se queda cerrada sobre el tejido. Sus mandíbulas terminan en varios dientes finos que encajan entre sí (4 × 5 en el modelo estándar). Sirve para tomar y mantener sujetos tejidos y estructuras durante la operación. Mide de 14 a 20 cm.</t>
+          <t>Pinza de aprehensión con anillos y cremallera, que se queda cerrada sobre el tejido. Sus mandíbulas terminan en una hilera de dientes cortos y finos que encajan entre sí (4 × 5 en el modelo estándar). Sirve para tomar y mantener sujetos tejidos y estructuras durante la operación; aprieta menos que la pinza Kocher. Mide de 14 a 20 cm.</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>CICR, XSINMEDI500215, pinza de Allis: https://itemscatalogue.redcross.int/detail.aspx?itemcode=XSINMEDI500215&amp;from=kit
+          <t>CICR, XSINMEDI500, pinza de Allis: https://itemscatalogue.redcross.int/health--3/surgical-instruments--24/surgical-instruments--111/forceps-soft-tissue-serratedtoothed-allis--XSINMEDI500.aspx
+Open Exam Prep, HSPA CIS, 1.5 Clamping, Grasping &amp; Occluding Instruments: https://open-exam-prep.com/study-guides/hspa-cis/instrument-identification/clamping-grasping
 Sánchez-Sarría O. y otros, Manual de instrumental quirúrgico, Medisur 2014;12(5), p. 784: https://medisur.sld.cu/index.php/medisur/article/view/2662</t>
         </is>
       </c>
@@ -25097,14 +25103,15 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Pinza de aprehensión con anillos y cremallera suave. Su punta es ancha, redondeada y abierta en el centro (fenestrada), sin dientes, con estrías atraumáticas. Toma tejidos blandos y delicados, sobre todo el intestino, sin aplastarlos ni perforarlos. Es más suave con el tejido que la pinza de Allis. Mide de 16 a 21 cm.</t>
+          <t>Pinza de aprehensión atraumática, con anillos y cremallera suave. Su punta es ancha, curva y abierta en el centro (fenestrada), sin dientes: rodea y toma estructuras tubulares delicadas, como el intestino, sin aplastarlas. Mide de 16 a 21 cm.</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>UNICEF Supply Catalogue, S0736500, Babcock 200 mm (ref. KLS Martin 30 192 20): https://supply.unicef.org/s0736500.html
-KLS Martin, 30-196-20-07: https://www.klsmartin.com/shop/en/products/product/30-196-20-07/
-Eickemeyer, 145616: https://www.eickemeyer.com/shop/145616-intestinal-and-tissue-forceps-babcock-16-cm-atraumatic-13535</t>
+          <t>CICR, XSINMEDI5010, pinza de Babcock: https://itemscatalogue.redcross.int/health--3/surgical-instruments--24/surgical-instruments--111/forceps-soft-tissue-babcock--XSINMEDI5010.aspx
+Open Exam Prep, HSPA CIS, 1.5 Clamping, Grasping &amp; Occluding Instruments: https://open-exam-prep.com/study-guides/hspa-cis/instrument-identification/clamping-grasping
+Eickemeyer, 145616, Babcock 16 cm: https://www.eickemeyer.com/shop/145616-intestinal-and-tissue-forceps-babcock-16-cm-atraumatic-13535
+KLS Martin, 30-196-20-07, pinza intestinal según Babcock: https://www.klsmartin.com/shop/en/products/product/30-196-20-07/</t>
         </is>
       </c>
     </row>
@@ -25205,12 +25212,13 @@
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Pinza de un solo cuerpo, de resorte y sin cremallera, como la de disección sin garra, pero con dientes en la punta. Los dientes de las dos ramas encajan entre sí: uno en una rama entre dos de la otra («1 × 2»). Así agarra con más firmeza que la sin garra. Mide de 14 a 20 cm.</t>
+          <t>Pinza de un solo cuerpo, de resorte y sin cremallera, como la de disección sin garra, pero con dientes en la punta que encajan entre sí: uno en una rama entre dos de la otra («1 × 2»). Los dientes agarran el tejido con firmeza y poca presión; se usa en tejidos como la piel. Mide de 14 a 20 cm.</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>CICR, XSINMEDI060020, pinza de disección 1 × 2 dientes (XSINMEDI060520): https://itemscatalogue.redcross.int/detail.aspx?itemcode=XSINMEDI060020&amp;from=kit
+          <t>CICR, XSINMEDI060, pinzas de disección con y sin dientes: https://itemscatalogue.redcross.int/health--3/surgical-instruments--24/surgical-instruments--111/forceps-dressing-standard-serrated-toothed--XSINMEDI060.aspx
+ErgoDenta, Tissue &amp; Dressing Forceps: https://ergodenta.dk/blog/products-13/tissue-dressing-forceps-adson-gerald-semken-allis-147
 Sánchez-Sarría O. y otros, Manual de instrumental quirúrgico, Medisur 2014;12(5), p. 784: https://medisur.sld.cu/index.php/medisur/article/view/2662
 UNAM, Facultad de Medicina, Práctica 3: estuche de disección (2023): https://anatomia.facmed.unam.mx/wp-content/uploads/2023/10/Practica-3-estuche-2023-2024.pdf</t>
         </is>
@@ -25229,12 +25237,13 @@
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Pinza de un solo cuerpo, de resorte: se cierra al presionar sus ramas y se abre sola al soltarlas. No tiene cremallera. Sus puntas son estriadas y no tienen dientes, por eso no lastiman el tejido. Sirve para tomar tejidos delicados durante la disección y la sutura, y para manipular gasas y apósitos. Mide de 14,5 a 20 cm.</t>
+          <t>Pinza de un solo cuerpo, de resorte y sin cremallera: se cierra al presionar sus ramas y se abre al soltarlas. Sus puntas son estriadas y no tienen dientes, así que toma tejido delicado, gasas y suturas sin dañarlos. También sirve para tomar tejidos durante la disección y para coagular vasos. Mide de 14,5 a 20 cm.</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>CICR, XSINMEDI060020, pinza de disección con o sin dientes: https://itemscatalogue.redcross.int/detail.aspx?itemcode=XSINMEDI060020&amp;from=kit
+          <t>CICR, XSINMEDI060, pinzas de disección con y sin dientes: https://itemscatalogue.redcross.int/health--3/surgical-instruments--24/surgical-instruments--111/forceps-dressing-standard-serrated-toothed--XSINMEDI060.aspx
+ErgoDenta, Tissue &amp; Dressing Forceps: https://ergodenta.dk/blog/products-13/tissue-dressing-forceps-adson-gerald-semken-allis-147
 Sánchez-Sarría O. y otros, Manual de instrumental quirúrgico, Medisur 2014;12(5), p. 784: https://medisur.sld.cu/index.php/medisur/article/view/2662
 UNAM, Facultad de Medicina, Práctica 3: estuche de disección (2023): https://anatomia.facmed.unam.mx/wp-content/uploads/2023/10/Practica-3-estuche-2023-2024.pdf</t>
         </is>
@@ -25301,16 +25310,16 @@
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>Pinza hemostática con anillos y cremallera, recta o curva, de unos 14 cm. Sus mandíbulas tienen estrías transversales solo en la mitad de la punta; eso la distingue de la pinza Crile, que es estriada en toda la mandíbula. Sirve para pinzar vasos o tejidos y así evitar la hemorragia.</t>
+          <t>Pinza hemostática con anillos y cremallera, recta o curva, de unos 14 cm. Sus mandíbulas no tienen dientes y sus estrías transversales llegan solo a la mitad, desde la punta; eso la distingue de la pinza Crile, estriada en toda la mandíbula. Sirve para pinzar vasos o tejidos y así evitar la hemorragia.</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
           <t>UNAM, Facultad de Medicina, Práctica 3: estuche de disección (2023): https://anatomia.facmed.unam.mx/wp-content/uploads/2023/10/Practica-3-estuche-2023-2024.pdf
 Sánchez-Sarría O. y otros, Manual de instrumental quirúrgico, Medisur 2014;12(5), p. 784: https://medisur.sld.cu/index.php/medisur/article/view/2662
-MSF Unicat 14066, Kelly 14 cm: https://unicat.msf.org/cat/product/14066
-Remma, Kelly 14 cm: https://remma.fr/en/model/kelly-clamp-straight-curved-jaws-serrated-14-cm
-Medikabazaar, guía de la pinza Kelly: https://www.medikabazaar.com/blogs/kelly-forceps-types-uses-surgical-procurement-guide</t>
+Open Exam Prep, HSPA CIS, 1.5 Clamping, Grasping &amp; Occluding Instruments: https://open-exam-prep.com/study-guides/hspa-cis/instrument-identification/clamping-grasping
+Medikabazaar, guía de la pinza Kelly: https://www.medikabazaar.com/blogs/kelly-forceps-types-uses-surgical-procurement-guide
+MSF Unicat 14066, Kelly 14 cm: https://unicat.msf.org/cat/product/14066</t>
         </is>
       </c>
     </row>
@@ -25327,14 +25336,15 @@
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Pinza hemostática de Adson, con anillos y cremallera, recta o curva, de unos 18 cm. Sus ramas son más largas que las de la Kelly y sus mandíbulas, estriadas en parte. Sirve para pinzar vasos pequeños. No es la pinza de disección Adson, que es de aprehensión.</t>
+          <t>Pinza hemostática de Adson, recta o curva, de unos 18 a 19 cm, con anillos y cremallera como las demás pinzas de hemostasia. Sus mandíbulas, de unos 30 mm, son estriadas en sus dos tercios. No es la pinza de disección Adson, que es de aprehensión.</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>Sánchez-Sarría O. y otros, Manual de instrumental quirúrgico, Medisur 2014;12(5), p. 784: https://medisur.sld.cu/index.php/medisur/article/view/2662
-Sklar 50-1372, Adson hemostática recta, en McKesson: https://mms.mckesson.com/product/253068/Sklar-50-1372
-Sklar 50-1472, Adson hemostática curva, en McKesson: https://mms.mckesson.com/product/377086/Sklar-50-1472</t>
+          <t>Sánchez-Sarría O. y otros, Manual de instrumental quirúrgico, Medisur 2014;12(5), p. 783: https://medisur.sld.cu/index.php/medisur/article/view/2662
+Sánchez-Sarría O. y otros, Manual de instrumental quirúrgico, Medisur 2014;12(5), p. 784: https://medisur.sld.cu/index.php/medisur/article/view/2662
+Teleflex, Adson Hemostatic Forceps: https://us.myteleflex.com/en/USD/All-Categories/Surgical-Instruments/General/Adson-Hemostatic-Forceps/p/su-AdsonHemostaticForceps
+KLS Martin, 13-365-18-07, Haemostatic forceps acc. to Adson: https://www.klsmartin.com/shop/en/products/product/13-365-18-07</t>
         </is>
       </c>
     </row>
@@ -25351,12 +25361,13 @@
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>Pinza hemostática con anillos y cremallera, recta o curva, de 14 a 22 cm. Sus mandíbulas son estriadas y terminan en dientes (1 × 2: uno en una rama entre dos de la otra). Sirve para hemostasia, para sujetar tejidos y para sostener gasas.</t>
+          <t>Pinza hemostática con anillos y cremallera, recta o curva, de 14 a 22 cm. Sus mandíbulas tienen estrías marcadas y terminan en dientes que encajan entre sí (1 × 2: uno en una rama entre dos de la otra). Los dientes dan un agarre que no se resbala, para tejidos resistentes como la aponeurosis; por eso no se usa en tejido delicado. Sirve para hemostasia, para sujetar tejidos y para sostener gasas.</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>CICR, XSINMEDI161214, Kocher y R-Ochsner: https://itemscatalogue.redcross.int/detail.aspx?itemcode=XSINMEDI161214&amp;from=kit
+          <t>CICR, XSINMEDI16, Kocher y R-Ochsner: https://itemscatalogue.redcross.int/health--3/surgical-instruments--24/surgical-instruments--111/forceps-hemostatic-straightcurved-heavily-serrated-curved-kosher-r-ochsner-wertheim--XSINMEDI16.aspx
+Open Exam Prep, HSPA CIS, 1.5 Clamping, Grasping &amp; Occluding Instruments: https://open-exam-prep.com/study-guides/hspa-cis/instrument-identification/clamping-grasping
 Sánchez-Sarría O. y otros, Manual de instrumental quirúrgico, Medisur 2014;12(5), p. 786: https://medisur.sld.cu/index.php/medisur/article/view/2662</t>
         </is>
       </c>
@@ -25391,13 +25402,13 @@
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>Pinza larga y curva, de unos 22 a 23 cm, con anillos, hecha para tomar el conducto biliar. Sus mandíbulas son estriadas.</t>
+          <t>Pinza larga y curva, de unos 22 a 23 cm, con anillos y mandíbulas estriadas. En los catálogos aparece como pinza para el conducto biliar.</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
           <t>KLS Martin, 13-671-23-07, bile duct forceps acc. to Moynihan: https://www.klsmartin.com/shop/en/products/product/13-671-23-07/
-Ambler Surgical 32-444, registro FDA (UDI 00190660066611): https://beudamed.com/fda_udis/00190660066611</t>
+Ambler Surgical 32-444, registro GUDID (FDA): https://accessgudid.nlm.nih.gov/devices/00190660066611</t>
         </is>
       </c>
     </row>
@@ -25414,12 +25425,13 @@
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>Pinza hemostática pequeña y delgada (de Halsted), de unos 12,5 cm, con anillos y cremallera. Sus mandíbulas son finas y curvas. Sirve para pinzar vasos pequeños, para disecciones finas y para tomar tejidos delicados.</t>
+          <t>Pinza hemostática pequeña y delgada (de Halsted), de unos 12,5 cm, con anillos y cremallera. Es la más pequeña y fina de las pinzas hemostáticas, de mandíbulas finas y curvas. Sirve para pinzar vasos pequeños, para disecciones finas y para tomar tejidos delicados.</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>CICR, XSINMEDI154512, H-Mosquito curva: https://itemscatalogue.redcross.int/detail.aspx?itemcode=XSINMEDI154512&amp;from=kit
+          <t>CICR, XSINMEDI154, H-Mosquito: https://itemscatalogue.redcross.int/health--3/surgical-instruments--24/surgical-instruments--111/forceps-hemostatic-curvedstraight-serratedtoothed-h-mosquito--XSINMEDI154.aspx
+Open Exam Prep, HSPA CIS, 1.5 Clamping, Grasping &amp; Occluding Instruments: https://open-exam-prep.com/study-guides/hspa-cis/instrument-identification/clamping-grasping
 UNAM, Facultad de Medicina, Práctica 3: estuche de disección (2023): https://anatomia.facmed.unam.mx/wp-content/uploads/2023/10/Practica-3-estuche-2023-2024.pdf
 Sánchez-Sarría O. y otros, Manual de instrumental quirúrgico, Medisur 2014;12(5), p. 784: https://medisur.sld.cu/index.php/medisur/article/view/2662</t>
         </is>
@@ -25450,12 +25462,14 @@
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>Pinza hemostática grande y fuerte (Rochester-Péan), con anillos y cremallera, recta o curva, de 16 a 26 cm. Sus mandíbulas tienen estrías transversales en todo su largo. Sirve para pinzar tejidos gruesos y vasos grandes.</t>
+          <t>Pinza hemostática grande y fuerte (Rochester-Péan), con anillos y cremallera, recta o curva, de 16 a 26 cm. Sus mandíbulas no tienen dientes y tienen estrías transversales en todo su largo. Sirve para pinzar tejidos y vasos grandes, y para tomar y disecar estructuras profundas.</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>Sánchez-Sarría O. y otros, Manual de instrumental quirúrgico, Medisur 2014;12(5), p. 784: https://medisur.sld.cu/index.php/medisur/article/view/2662
+          <t>CICR, XSINMEDI161, Rochester-Pean: https://itemscatalogue.redcross.int/health--3/surgical-instruments--24/surgical-instruments--111/forceps-hemostatic-straightcurved-serrated-rochester-pean--XSINMEDI161.aspx
+Open Exam Prep, HSPA CIS, 1.5 Clamping, Grasping &amp; Occluding Instruments: https://open-exam-prep.com/study-guides/hspa-cis/instrument-identification/clamping-grasping
+Sánchez-Sarría O. y otros, Manual de instrumental quirúrgico, Medisur 2014;12(5), p. 784: https://medisur.sld.cu/index.php/medisur/article/view/2662
 MSF Unicat 14060, R-Pean 16 cm: https://unicat.msf.org/cat/product/14060
 Covetrus, Rochester-Pean: https://products.covetrus.com/surgical-instruments/forceps-hemostats/hemostat-forceps-rochester-pean
 UNFPA, 1000326, Rochester-Pean 22 cm: https://globalsupply.unfpa.org/products/forceps-artery-rochester-pean-22cm-straight-1000326.html</t>
@@ -25511,12 +25525,12 @@
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>Portaagujas (Mayo-Hegar) con anillos y cremallera: sostiene la aguja mientras se sutura. Sus mandíbulas tienen estrías marcadas, para agujas estándar, y una ranura a lo largo que evita dañar la aguja. La cremallera deja ajustar la presión. El largo mide de 18 a 23 cm; el corriente, 15 cm.</t>
+          <t>Portaagujas con anillos y cremallera: sostiene la aguja mientras se sutura. En el modelo Mayo-Hegar, para agujas estándar, sus mandíbulas tienen estrías marcadas y una ranura a lo largo que evita dañar la aguja; la cremallera deja ajustar la presión. Se fabrica de 15 a 23 cm.</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>CICR, XSINMEDI101815, portaagujas Mayo-Hegar: https://itemscatalogue.redcross.int/detail.aspx?itemcode=XSINMEDI101815&amp;from=kit
+          <t>CICR, XSINMEDI101, portaagujas Mayo-Hegar: https://itemscatalogue.redcross.int/health--3/surgical-instruments--24/surgical-instruments--111/needle-holder-mayo-hegar-baby-crile-stevens-barraquer--XSINMEDI101.aspx
 Sánchez-Sarría O. y otros, Manual de instrumental quirúrgico, Medisur 2014;12(5), p. 784: https://medisur.sld.cu/index.php/medisur/article/view/2662</t>
         </is>
       </c>
@@ -25654,12 +25668,12 @@
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>Separador manual, de un solo cuerpo, de doble extremo: en cada punta tiene una lámina plana doblada en ángulo recto, de distinto tamaño (24 × 16 y 28 × 16 mm). Mide unos 15 cm y se usa en pares. Retrae la piel, el tejido subcutáneo y el músculo para que el cirujano vea el campo operatorio.</t>
+          <t>Separador manual, de un solo cuerpo y doble extremo: en cada punta tiene una lámina doblada en ángulo, de distinto tamaño (24 × 16 y 28 × 16 mm). Mide unos 15 cm y viene en pares. Retrae la piel, el tejido subcutáneo y el músculo para que el cirujano vea el campo operatorio.</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>CICR, XSINMEDI221015, Farabeuf: https://itemscatalogue.redcross.int/health--3/surgical-instruments--24/surgical-instruments--111/retractor-general-double-ended-farabeuf-roux-senn-miller--XSINMEDI200.aspx
+          <t>CICR, XSINMEDI200, separadores Farabeuf (XSINMEDI221015) y Senn-Miller (XSINMEDI200509): https://itemscatalogue.redcross.int/health--3/surgical-instruments--24/surgical-instruments--111/retractor-general-double-ended-farabeuf-roux-senn-miller--XSINMEDI200.aspx
 UNAM, Facultad de Medicina, Práctica 3: estuche de disección (2023): https://anatomia.facmed.unam.mx/wp-content/uploads/2023/10/Practica-3-estuche-2023-2024.pdf
 Sánchez-Sarría O. y otros, Manual de instrumental quirúrgico, Medisur 2014;12(5), p. 783: https://medisur.sld.cu/index.php/medisur/article/view/2662</t>
         </is>
@@ -25690,14 +25704,12 @@
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>Separador manual pequeño, de doble extremo: en un extremo tiene tres puntas curvas (romas o agudas) y en el otro, una lámina delgada doblada. Mide unos 15 a 16 cm. Retrae la piel, el tejido o el músculo en sitios quirúrgicos pequeños.</t>
+          <t>Separador manual pequeño, de doble extremo: en un extremo tiene tres puntas romas y curvas, y en el otro, una lámina delgada doblada en ángulo. Mide unos 16 cm. Retrae la piel, el tejido subcutáneo o el músculo.</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>CICR, XSINMEDI200509, Senn-Miller: https://itemscatalogue.redcross.int/health--3/surgical-instruments--24/surgical-instruments--111/retractor-general-double-ended-farabeuf-roux-senn-miller--XSINMEDI200.aspx
-Sklar, Miller-Senn, en VWR: https://b2b-pr.vwr.com/store/product/18360095/null
-Sklar Senn, en Ward's Science: https://www.wardsci.com/us/en/product/NA1063474/senn-retractor-or-grade-sklar
+          <t>CICR, XSINMEDI200, separadores Farabeuf (XSINMEDI221015) y Senn-Miller (XSINMEDI200509): https://itemscatalogue.redcross.int/health--3/surgical-instruments--24/surgical-instruments--111/retractor-general-double-ended-farabeuf-roux-senn-miller--XSINMEDI200.aspx
 Sánchez-Sarría O. y otros, Manual de instrumental quirúrgico, Medisur 2014;12(5), p. 783: https://medisur.sld.cu/index.php/medisur/article/view/2662</t>
         </is>
       </c>
@@ -25979,13 +25991,14 @@
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>Hoja de bisturí pequeña, de acero, con el filo curvo, que se monta en los mangos N.° 3 y N.° 7. Es la forma clásica para las incisiones en piel y músculo.</t>
+          <t>Hoja de bisturí pequeña, de filo curvo, que se monta en los mangos N.° 3 y N.° 7. Es una de las formas clásicas: sirve para incisiones de distinto tamaño en piel y músculo.</t>
         </is>
       </c>
       <c r="E105" t="inlineStr">
         <is>
           <t>Sánchez-Sarría O. y otros, Manual de instrumental quirúrgico, Medisur 2014;12(5), p. 783: https://medisur.sld.cu/index.php/medisur/article/view/2662
-Swann-Morton, hojas de bisturí (IMS Euro): https://imseuro.co.uk/swann-mortonr-scalpel-blades</t>
+Swann-Morton N.° 10, en Scientific Laboratory Supplies: https://scientificlabs.co.uk/product/scalpels-and-blades/INS4670
+Open Exam Prep, HSPA CIS, 1.4 Cutting &amp; Dissecting Instruments: https://open-exam-prep.com/study-guides/hspa-cis/instrument-identification/cutting-dissecting</t>
         </is>
       </c>
     </row>
@@ -26002,13 +26015,15 @@
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>Hojas pequeñas N.° 10 y N.° 11, que se montan en el mango N.° 3. La N.° 10 tiene el filo curvo y es la forma clásica para incisiones en piel y músculo. La N.° 11 es triangular, con la punta aguda y el filo en uno de sus lados largos: sirve para incisiones punzantes, como abrir un absceso o el sitio de un dren.</t>
+          <t>Hojas pequeñas N.° 10 y N.° 11, que se montan en el mango N.° 3. La N.° 10 tiene el filo curvo y sirve para incisiones en piel y músculo. La N.° 11 es triangular y alargada, con la punta aguda y el filo en su lado más largo: sirve para incisiones punzantes, como abrir un absceso o el sitio de un dren.</t>
         </is>
       </c>
       <c r="E106" t="inlineStr">
         <is>
           <t>Sánchez-Sarría O. y otros, Manual de instrumental quirúrgico, Medisur 2014;12(5), p. 783: https://medisur.sld.cu/index.php/medisur/article/view/2662
-Swann-Morton, hojas de bisturí (IMS Euro): https://imseuro.co.uk/swann-mortonr-scalpel-blades</t>
+Swann-Morton N.° 10, en Scientific Laboratory Supplies: https://scientificlabs.co.uk/product/scalpels-and-blades/INS4670
+Swann-Morton N.° 11, en Scientific Laboratory Supplies: https://scientificlabs.co.uk/product/scalpels-and-blades/INS4674
+Buckner B., Scalpels, Journal of Medical Insight (JOMI) 300.1, 2023, doi:10.24296/jomi/300.1: https://jomi.com/article/300.1/scalpels/transcript</t>
         </is>
       </c>
     </row>
@@ -26037,13 +26052,14 @@
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>Hoja de bisturí pequeña, con el filo curvo y corto, que se monta en los mangos N.° 3 y N.° 7. Es la forma más usada para incisiones cortas y precisas.</t>
+          <t>Hoja de bisturí pequeña, con el filo curvo y corto, que se monta en los mangos N.° 3 y N.° 7. Es la forma más usada para incisiones cortas y precisas, como quitar una lesión de la piel.</t>
         </is>
       </c>
       <c r="E108" t="inlineStr">
         <is>
           <t>Sánchez-Sarría O. y otros, Manual de instrumental quirúrgico, Medisur 2014;12(5), p. 783: https://medisur.sld.cu/index.php/medisur/article/view/2662
-Swann-Morton, hojas de bisturí (IMS Euro): https://imseuro.co.uk/swann-mortonr-scalpel-blades</t>
+Swann-Morton N.° 15, en Scientific Laboratory Supplies: https://scientificlabs.co.uk/product/scalpels-and-blades/INS4678
+Buckner B., Scalpels, Journal of Medical Insight (JOMI) 300.1, 2023, doi:10.24296/jomi/300.1: https://jomi.com/article/300.1/scalpels/transcript</t>
         </is>
       </c>
     </row>
@@ -26060,14 +26076,14 @@
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>Hoja de bisturí grande, que se monta en el mango N.° 4. Es como una N.° 10 de mayor tamaño: filo curvo y lomo recto sin filo.</t>
+          <t>Hoja de bisturí grande, que se monta en el mango N.° 4. Es como una N.° 10 de mayor tamaño: filo curvo y lomo plano sin filo. Sirve para las incisiones grandes.</t>
         </is>
       </c>
       <c r="E109" t="inlineStr">
         <is>
           <t>Sánchez-Sarría O. y otros, Manual de instrumental quirúrgico, Medisur 2014;12(5), p. 783: https://medisur.sld.cu/index.php/medisur/article/view/2662
-CICR, set KMSISBAS01, mango N.° 4 para hojas 20: https://itemscatalogue.redcross.int/detail.aspx?itemcode=KMSISBAS01&amp;from=kit
-Swann-Morton N.° 20, en Scientific Laboratory Supplies: https://scientificlabs.co.uk/product/scalpels-and-blades/INS4680</t>
+Swann-Morton N.° 20, en Scientific Laboratory Supplies: https://scientificlabs.co.uk/product/scalpels-and-blades/INS4680
+Buckner B., Scalpels, Journal of Medical Insight (JOMI) 300.1, 2023, doi:10.24296/jomi/300.1: https://jomi.com/article/300.1/scalpels/transcript</t>
         </is>
       </c>
     </row>
@@ -26264,14 +26280,14 @@
       </c>
       <c r="D125" t="inlineStr">
         <is>
-          <t>Pinza de tracción con anillos y cremallera. Sus puntas son curvas y tienen tres dientes agudos en cada rama (3 × 3), que penetran el tejido fibroso para que el agarre no se suelte. Se usa para tomar y traccionar el tejido y la glándula en la cirugía de tiroides, y el tejido mamario en la mastectomía. Mide unos 15 a 16 cm.</t>
+          <t>Pinza de Lahey para bocio, con anillos y cremallera, de unos 15 cm. Sujeta y tracciona el tejido firme de la glándula tiroides durante la tiroidectomía. Se fabrica en dos versiones: con tres dientes en cada rama (3 × 3) o con mandíbulas curvas de estrías transversales.</t>
         </is>
       </c>
       <c r="E125" t="inlineStr">
         <is>
-          <t>Sklar 17-3562, en McKesson: https://mms.mckesson.com/product/375723/Sklar-17-3562
-Aspen Surgical 73-7233, Lahey Goiter Traction 3x3: https://www.mymapmedical.com/shop/aspen-surgical-73-7233-180067
-Integra Miltex 7-62, en McKesson: https://mms.mckesson.com/product/263612/Integra-Lifesciences-7-62</t>
+          <t>Aspen Surgical 73-7233, Lahey Goiter Traction 3x3, registro GUDID (FDA): https://accessgudid.nlm.nih.gov/devices/00887482040065
+NPrep, AIIMS Delhi 2019, pinza de Lahey: https://nprep.in/question-answer/the-following-instrument-is-used-in-which-surgery-ZMAstWpZR9WCkGj4WTtq8
+Sánchez-Sarría O. y otros, Manual de instrumental quirúrgico, Medisur 2014;12(5), p. 783: https://medisur.sld.cu/index.php/medisur/article/view/2662</t>
         </is>
       </c>
     </row>
@@ -26444,12 +26460,13 @@
       </c>
       <c r="D139" t="inlineStr">
         <is>
-          <t>Tijera fuerte, de hojas gruesas y puntas romas, recta o curva, de 15 a 23 cm. Corta por cizalla. La recta se usa para cortar suturas, gasas y otros materiales; la curva también corta tejido que no es delicado.</t>
+          <t>Tijera de hojas fuertes y relativamente cortas, con puntas romas, recta o curva, de 15 a 23 cm. Corta por cizalla. La recta se usa para cortar suturas y apósitos; la curva, para cortar tejido resistente, como la aponeurosis.</t>
         </is>
       </c>
       <c r="E139" t="inlineStr">
         <is>
-          <t>CICR, XSINMEDI035117, tijera de Mayo: https://itemscatalogue.redcross.int/detail.aspx?itemcode=XSINMEDI035117&amp;from=kit
+          <t>CICR, XSINMEDI035, tijera de Mayo: https://itemscatalogue.redcross.int/health--3/surgical-instruments--24/surgical-instruments--111/scissors-basic-dissecting-straightcurved-blunt-mayo--XSINMEDI035.aspx
+Open Exam Prep, HSPA CIS, 1.4 Cutting &amp; Dissecting Instruments: https://open-exam-prep.com/study-guides/hspa-cis/instrument-identification/cutting-dissecting
 Sánchez-Sarría O. y otros, Manual de instrumental quirúrgico, Medisur 2014;12(5), p. 783: https://medisur.sld.cu/index.php/medisur/article/view/2662</t>
         </is>
       </c>
@@ -26467,12 +26484,13 @@
       </c>
       <c r="D140" t="inlineStr">
         <is>
-          <t>Tijera delgada, de puntas romas, casi siempre curva, de 14 a 23 cm. Es la tijera para la disección fina de los tejidos; el material (suturas, gasas) se corta con la tijera de Mayo.</t>
+          <t>Tijera delgada, de puntas romas, curva o recta, de 14 a 23 cm: ramas largas y hojas cortas y finas. Es la tijera para la disección fina de los tejidos. No se usa para cortar suturas, porque eso la desafila; el material se corta con la tijera de Mayo.</t>
         </is>
       </c>
       <c r="E140" t="inlineStr">
         <is>
-          <t>CICR, XSINMEDI043318, tijera de Metzenbaum: https://itemscatalogue.redcross.int/detail.aspx?itemcode=XSINMEDI043318&amp;from=kit
+          <t>CICR, XSINMEDI043, tijera de Metzenbaum: https://itemscatalogue.redcross.int/health--3/surgical-instruments--24/surgical-instruments--111/scissors-dissection-straightcurved-blunt-metzenbaum--XSINMEDI043.aspx
+Open Exam Prep, HSPA CIS, 1.4 Cutting &amp; Dissecting Instruments: https://open-exam-prep.com/study-guides/hspa-cis/instrument-identification/cutting-dissecting
 Sánchez-Sarría O. y otros, Manual de instrumental quirúrgico, Medisur 2014;12(5), p. 783: https://medisur.sld.cu/index.php/medisur/article/view/2662</t>
         </is>
       </c>

</xml_diff>